<commit_message>
chore: calibra a base de clientes e as metas do gerador
A base crescia rápido demais (receita +71% no ano), o que fazia todos
os vendedores baterem a meta com folga. Clientes passam a ter
histórico desde 2016 com churn de 50%, a tendência de frequência cai
para 2% ao ano e as metas de 2025 sobem para +20% sobre 2024. Resultado:
receita +21%, atingimento anual entre 63% e 148%. Dados regenerados.
</commit_message>
<xml_diff>
--- a/data/raw/metas_2025.xlsx
+++ b/data/raw/metas_2025.xlsx
@@ -513,43 +513,43 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>422000</v>
+        <v>207000</v>
       </c>
       <c r="D4" t="n">
-        <v>399000</v>
+        <v>167000</v>
       </c>
       <c r="E4" t="n">
-        <v>446000</v>
+        <v>282000</v>
       </c>
       <c r="F4" t="n">
-        <v>383000</v>
+        <v>372000</v>
       </c>
       <c r="G4" t="n">
-        <v>379000</v>
+        <v>471000</v>
       </c>
       <c r="H4" t="n">
-        <v>343000</v>
+        <v>314000</v>
       </c>
       <c r="I4" t="n">
-        <v>318000</v>
+        <v>345000</v>
       </c>
       <c r="J4" t="n">
-        <v>492000</v>
+        <v>340000</v>
       </c>
       <c r="K4" t="n">
-        <v>582000</v>
+        <v>477000</v>
       </c>
       <c r="L4" t="n">
-        <v>503000</v>
+        <v>336000</v>
       </c>
       <c r="M4" t="n">
-        <v>838000</v>
+        <v>298000</v>
       </c>
       <c r="N4" t="n">
-        <v>537000</v>
+        <v>515000</v>
       </c>
       <c r="O4" t="n">
-        <v>5642000</v>
+        <v>4124000</v>
       </c>
     </row>
     <row r="5">
@@ -565,66 +565,66 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>R$ 548.000,00</t>
+          <t>R$ 229.000,00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>R$ 366.000,00</t>
+          <t>R$ 441.000,00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>R$ 456.000,00</t>
+          <t>R$ 301.000,00</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>R$ 286.000,00</t>
+          <t>R$ 252.000,00</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>R$ 380.000,00</t>
+          <t>R$ 205.000,00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>R$ 432.000,00</t>
+          <t>R$ 358.000,00</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>R$ 544.000,00</t>
+          <t>R$ 282.000,00</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>R$ 312.000,00</t>
+          <t>R$ 233.000,00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>R$ 296.000,00</t>
+          <t>R$ 297.000,00</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>R$ 372.000,00</t>
+          <t>R$ 280.000,00</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>R$ 381.000,00</t>
+          <t>R$ 538.000,00</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>R$ 444.000,00</t>
+          <t>R$ 398.000,00</t>
         </is>
       </c>
       <c r="O5" t="n">
-        <v>4817000</v>
+        <v>3814000</v>
       </c>
     </row>
     <row r="6">
@@ -639,43 +639,43 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>296000</v>
+        <v>133000</v>
       </c>
       <c r="D6" t="n">
-        <v>171000</v>
+        <v>193000</v>
       </c>
       <c r="E6" t="n">
-        <v>282000</v>
+        <v>159000</v>
       </c>
       <c r="F6" t="n">
+        <v>117000</v>
+      </c>
+      <c r="G6" t="n">
+        <v>143000</v>
+      </c>
+      <c r="H6" t="n">
+        <v>119000</v>
+      </c>
+      <c r="I6" t="n">
+        <v>104000</v>
+      </c>
+      <c r="J6" t="n">
+        <v>135000</v>
+      </c>
+      <c r="K6" t="n">
+        <v>154000</v>
+      </c>
+      <c r="L6" t="n">
         <v>167000</v>
       </c>
-      <c r="G6" t="n">
-        <v>189000</v>
-      </c>
-      <c r="H6" t="n">
-        <v>199000</v>
-      </c>
-      <c r="I6" t="n">
-        <v>189000</v>
-      </c>
-      <c r="J6" t="n">
-        <v>248000</v>
-      </c>
-      <c r="K6" t="n">
-        <v>217000</v>
-      </c>
-      <c r="L6" t="n">
-        <v>198000</v>
-      </c>
       <c r="M6" t="n">
-        <v>261000</v>
+        <v>115000</v>
       </c>
       <c r="N6" t="n">
-        <v>265000</v>
+        <v>262000</v>
       </c>
       <c r="O6" t="n">
-        <v>2682000</v>
+        <v>1801000</v>
       </c>
     </row>
     <row r="7">
@@ -691,66 +691,66 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>R$ 141.000,00</t>
+          <t>R$ 364.000,00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>R$ 262.000,00</t>
+          <t>R$ 391.000,00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>R$ 229.000,00</t>
+          <t>R$ 279.000,00</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>R$ 264.000,00</t>
+          <t>R$ 310.000,00</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>R$ 329.000,00</t>
+          <t>R$ 413.000,00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>R$ 265.000,00</t>
+          <t>R$ 294.000,00</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>R$ 294.000,00</t>
+          <t>R$ 247.000,00</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>R$ 257.000,00</t>
+          <t>R$ 387.000,00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>R$ 225.000,00</t>
+          <t>R$ 272.000,00</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>R$ 363.000,00</t>
+          <t>R$ 155.000,00</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>R$ 437.000,00</t>
+          <t>R$ 296.000,00</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>R$ 450.000,00</t>
+          <t>R$ 211.000,00</t>
         </is>
       </c>
       <c r="O7" t="n">
-        <v>3516000</v>
+        <v>3619000</v>
       </c>
     </row>
     <row r="8">
@@ -765,43 +765,43 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>338000</v>
+        <v>289000</v>
       </c>
       <c r="D8" t="n">
-        <v>321000</v>
+        <v>263000</v>
       </c>
       <c r="E8" t="n">
-        <v>204000</v>
+        <v>182000</v>
       </c>
       <c r="F8" t="n">
-        <v>302000</v>
+        <v>253000</v>
       </c>
       <c r="G8" t="n">
+        <v>262000</v>
+      </c>
+      <c r="H8" t="n">
+        <v>190000</v>
+      </c>
+      <c r="I8" t="n">
+        <v>292000</v>
+      </c>
+      <c r="J8" t="n">
+        <v>314000</v>
+      </c>
+      <c r="K8" t="n">
+        <v>228000</v>
+      </c>
+      <c r="L8" t="n">
+        <v>337000</v>
+      </c>
+      <c r="M8" t="n">
+        <v>394000</v>
+      </c>
+      <c r="N8" t="n">
         <v>279000</v>
       </c>
-      <c r="H8" t="n">
-        <v>311000</v>
-      </c>
-      <c r="I8" t="n">
-        <v>313000</v>
-      </c>
-      <c r="J8" t="n">
-        <v>392000</v>
-      </c>
-      <c r="K8" t="n">
-        <v>465000</v>
-      </c>
-      <c r="L8" t="n">
-        <v>297000</v>
-      </c>
-      <c r="M8" t="n">
-        <v>466000</v>
-      </c>
-      <c r="N8" t="n">
-        <v>622000</v>
-      </c>
       <c r="O8" t="n">
-        <v>4310000</v>
+        <v>3283000</v>
       </c>
     </row>
     <row r="9">
@@ -817,66 +817,66 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>R$ 360.000,00</t>
+          <t>R$ 495.000,00</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>R$ 301.000,00</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>R$ 425.000,00</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>R$ 357.000,00</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>R$ 540.000,00</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>R$ 302.000,00</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>R$ 405.000,00</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>R$ 460.000,00</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>R$ 533.000,00</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
           <t>R$ 386.000,00</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>R$ 426.000,00</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>R$ 419.000,00</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>R$ 388.000,00</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>R$ 416.000,00</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>R$ 346.000,00</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>R$ 452.000,00</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>R$ 429.000,00</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>R$ 505.000,00</t>
-        </is>
-      </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>R$ 543.000,00</t>
+          <t>R$ 560.000,00</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>R$ 635.000,00</t>
+          <t>R$ 566.000,00</t>
         </is>
       </c>
       <c r="O9" t="n">
-        <v>5305000</v>
+        <v>5330000</v>
       </c>
     </row>
     <row r="10">
@@ -891,22 +891,22 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>419000</v>
+        <v>257000</v>
       </c>
       <c r="D10" t="n">
-        <v>432000</v>
+        <v>235000</v>
       </c>
       <c r="E10" t="n">
-        <v>332000</v>
+        <v>247000</v>
       </c>
       <c r="F10" t="n">
-        <v>664000</v>
+        <v>218000</v>
       </c>
       <c r="G10" t="n">
-        <v>476000</v>
+        <v>237000</v>
       </c>
       <c r="H10" t="n">
-        <v>407000</v>
+        <v>228000</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -915,7 +915,7 @@
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="n">
-        <v>2730000</v>
+        <v>1422000</v>
       </c>
     </row>
     <row r="11">
@@ -931,66 +931,66 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>R$ 281.000,00</t>
+          <t>R$ 165.000,00</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>R$ 188.000,00</t>
+          <t>R$ 104.000,00</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>R$ 299.000,00</t>
+          <t>R$ 149.000,00</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>R$ 347.000,00</t>
+          <t>R$ 119.000,00</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>R$ 222.000,00</t>
+          <t>R$ 138.000,00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>R$ 182.000,00</t>
+          <t>R$ 97.000,00</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>R$ 173.000,00</t>
+          <t>R$ 155.000,00</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>R$ 407.000,00</t>
+          <t>R$ 178.000,00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>R$ 290.000,00</t>
+          <t>R$ 120.000,00</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>R$ 363.000,00</t>
+          <t>R$ 142.000,00</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>R$ 319.000,00</t>
+          <t>R$ 193.000,00</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>R$ 412.000,00</t>
+          <t>R$ 184.000,00</t>
         </is>
       </c>
       <c r="O11" t="n">
-        <v>3483000</v>
+        <v>1744000</v>
       </c>
     </row>
     <row r="12">
@@ -1005,43 +1005,43 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>161000</v>
+        <v>385000</v>
       </c>
       <c r="D12" t="n">
-        <v>167000</v>
+        <v>341000</v>
       </c>
       <c r="E12" t="n">
-        <v>239000</v>
+        <v>370000</v>
       </c>
       <c r="F12" t="n">
-        <v>393000</v>
+        <v>386000</v>
       </c>
       <c r="G12" t="n">
-        <v>238000</v>
+        <v>398000</v>
       </c>
       <c r="H12" t="n">
-        <v>287000</v>
+        <v>187000</v>
       </c>
       <c r="I12" t="n">
-        <v>312000</v>
+        <v>358000</v>
       </c>
       <c r="J12" t="n">
-        <v>284000</v>
+        <v>307000</v>
       </c>
       <c r="K12" t="n">
-        <v>215000</v>
+        <v>298000</v>
       </c>
       <c r="L12" t="n">
-        <v>342000</v>
+        <v>306000</v>
       </c>
       <c r="M12" t="n">
-        <v>432000</v>
+        <v>428000</v>
       </c>
       <c r="N12" t="n">
-        <v>317000</v>
+        <v>336000</v>
       </c>
       <c r="O12" t="n">
-        <v>3387000</v>
+        <v>4100000</v>
       </c>
     </row>
     <row r="13">
@@ -1057,66 +1057,66 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>R$ 169.000,00</t>
+          <t>R$ 313.000,00</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>R$ 119.000,00</t>
+          <t>R$ 338.000,00</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>R$ 286.000,00</t>
+          <t>R$ 324.000,00</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>R$ 173.000,00</t>
+          <t>R$ 407.000,00</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>R$ 132.000,00</t>
+          <t>R$ 225.000,00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>R$ 211.000,00</t>
+          <t>R$ 304.000,00</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>R$ 467.000,00</t>
+          <t>R$ 224.000,00</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>R$ 201.000,00</t>
+          <t>R$ 279.000,00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>R$ 204.000,00</t>
+          <t>R$ 249.000,00</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>R$ 122.000,00</t>
+          <t>R$ 260.000,00</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>R$ 347.000,00</t>
+          <t>R$ 294.000,00</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>R$ 302.000,00</t>
+          <t>R$ 403.000,00</t>
         </is>
       </c>
       <c r="O13" t="n">
-        <v>2733000</v>
+        <v>3620000</v>
       </c>
     </row>
     <row r="14">
@@ -1131,43 +1131,43 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>175000</v>
+        <v>284000</v>
       </c>
       <c r="D14" t="n">
-        <v>116000</v>
+        <v>276000</v>
       </c>
       <c r="E14" t="n">
-        <v>77000</v>
+        <v>325000</v>
       </c>
       <c r="F14" t="n">
-        <v>118000</v>
+        <v>287000</v>
       </c>
       <c r="G14" t="n">
-        <v>149000</v>
+        <v>162000</v>
       </c>
       <c r="H14" t="n">
-        <v>283000</v>
+        <v>368000</v>
       </c>
       <c r="I14" t="n">
-        <v>126000</v>
+        <v>181000</v>
       </c>
       <c r="J14" t="n">
-        <v>187000</v>
+        <v>231000</v>
       </c>
       <c r="K14" t="n">
-        <v>122000</v>
+        <v>217000</v>
       </c>
       <c r="L14" t="n">
-        <v>235000</v>
+        <v>242000</v>
       </c>
       <c r="M14" t="n">
-        <v>277000</v>
+        <v>394000</v>
       </c>
       <c r="N14" t="n">
-        <v>320000</v>
+        <v>253000</v>
       </c>
       <c r="O14" t="n">
-        <v>2185000</v>
+        <v>3220000</v>
       </c>
     </row>
     <row r="15">
@@ -1183,66 +1183,66 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>R$ 39.000,00</t>
+          <t>R$ 191.000,00</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>R$ 51.000,00</t>
+          <t>R$ 103.000,00</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>R$ 55.000,00</t>
+          <t>R$ 153.000,00</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>R$ 67.000,00</t>
+          <t>R$ 152.000,00</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>R$ 46.000,00</t>
+          <t>R$ 210.000,00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>R$ 56.000,00</t>
+          <t>R$ 103.000,00</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>R$ 63.000,00</t>
+          <t>R$ 161.000,00</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>R$ 107.000,00</t>
+          <t>R$ 172.000,00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>R$ 82.000,00</t>
+          <t>R$ 260.000,00</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>R$ 90.000,00</t>
+          <t>R$ 263.000,00</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>R$ 143.000,00</t>
+          <t>R$ 249.000,00</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>R$ 164.000,00</t>
+          <t>R$ 261.000,00</t>
         </is>
       </c>
       <c r="O15" t="n">
-        <v>963000</v>
+        <v>2278000</v>
       </c>
     </row>
     <row r="16">
@@ -1257,43 +1257,43 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>180000</v>
+        <v>261000</v>
       </c>
       <c r="D16" t="n">
-        <v>246000</v>
+        <v>268000</v>
       </c>
       <c r="E16" t="n">
-        <v>228000</v>
+        <v>207000</v>
       </c>
       <c r="F16" t="n">
-        <v>200000</v>
+        <v>295000</v>
       </c>
       <c r="G16" t="n">
-        <v>283000</v>
+        <v>210000</v>
       </c>
       <c r="H16" t="n">
-        <v>182000</v>
+        <v>146000</v>
       </c>
       <c r="I16" t="n">
-        <v>355000</v>
+        <v>240000</v>
       </c>
       <c r="J16" t="n">
-        <v>337000</v>
+        <v>240000</v>
       </c>
       <c r="K16" t="n">
-        <v>329000</v>
+        <v>225000</v>
       </c>
       <c r="L16" t="n">
-        <v>499000</v>
+        <v>241000</v>
       </c>
       <c r="M16" t="n">
-        <v>328000</v>
+        <v>298000</v>
       </c>
       <c r="N16" t="n">
-        <v>348000</v>
+        <v>418000</v>
       </c>
       <c r="O16" t="n">
-        <v>3515000</v>
+        <v>3049000</v>
       </c>
     </row>
     <row r="17">
@@ -1309,66 +1309,66 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>R$ 261.000,00</t>
+          <t>R$ 394.000,00</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>R$ 188.000,00</t>
+          <t>R$ 437.000,00</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>R$ 170.000,00</t>
+          <t>R$ 707.000,00</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>R$ 71.000,00</t>
+          <t>R$ 435.000,00</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>R$ 331.000,00</t>
+          <t>R$ 388.000,00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>R$ 237.000,00</t>
+          <t>R$ 349.000,00</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>R$ 203.000,00</t>
+          <t>R$ 462.000,00</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>R$ 172.000,00</t>
+          <t>R$ 476.000,00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>R$ 344.000,00</t>
+          <t>R$ 339.000,00</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>R$ 261.000,00</t>
+          <t>R$ 518.000,00</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>R$ 457.000,00</t>
+          <t>R$ 422.000,00</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>R$ 568.000,00</t>
+          <t>R$ 547.000,00</t>
         </is>
       </c>
       <c r="O17" t="n">
-        <v>3263000</v>
+        <v>5474000</v>
       </c>
     </row>
     <row r="18">
@@ -1383,43 +1383,43 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>103000</v>
+        <v>204000</v>
       </c>
       <c r="D18" t="n">
-        <v>319000</v>
+        <v>188000</v>
       </c>
       <c r="E18" t="n">
-        <v>220000</v>
+        <v>172000</v>
       </c>
       <c r="F18" t="n">
-        <v>211000</v>
+        <v>112000</v>
       </c>
       <c r="G18" t="n">
-        <v>241000</v>
+        <v>124000</v>
       </c>
       <c r="H18" t="n">
-        <v>100000</v>
+        <v>154000</v>
       </c>
       <c r="I18" t="n">
-        <v>323000</v>
+        <v>168000</v>
       </c>
       <c r="J18" t="n">
-        <v>221000</v>
+        <v>283000</v>
       </c>
       <c r="K18" t="n">
-        <v>221000</v>
+        <v>156000</v>
       </c>
       <c r="L18" t="n">
-        <v>303000</v>
+        <v>274000</v>
       </c>
       <c r="M18" t="n">
-        <v>420000</v>
+        <v>354000</v>
       </c>
       <c r="N18" t="n">
-        <v>283000</v>
+        <v>262000</v>
       </c>
       <c r="O18" t="n">
-        <v>2965000</v>
+        <v>2451000</v>
       </c>
     </row>
     <row r="19">
@@ -1435,66 +1435,66 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>R$ 138.000,00</t>
+          <t>R$ 257.000,00</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>R$ 85.000,00</t>
+          <t>R$ 740.000,00</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>R$ 121.000,00</t>
+          <t>R$ 432.000,00</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>R$ 80.000,00</t>
+          <t>R$ 409.000,00</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>R$ 157.000,00</t>
+          <t>R$ 476.000,00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>R$ 131.000,00</t>
+          <t>R$ 594.000,00</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>R$ 133.000,00</t>
+          <t>R$ 403.000,00</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>R$ 178.000,00</t>
+          <t>R$ 720.000,00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>R$ 259.000,00</t>
+          <t>R$ 577.000,00</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>R$ 196.000,00</t>
+          <t>R$ 426.000,00</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>R$ 466.000,00</t>
+          <t>R$ 516.000,00</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>R$ 505.000,00</t>
+          <t>R$ 761.000,00</t>
         </is>
       </c>
       <c r="O19" t="n">
-        <v>2449000</v>
+        <v>6311000</v>
       </c>
     </row>
     <row r="20">
@@ -1515,25 +1515,25 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
-        <v>296000</v>
+        <v>402000</v>
       </c>
       <c r="J20" t="n">
-        <v>415000</v>
+        <v>323000</v>
       </c>
       <c r="K20" t="n">
-        <v>297000</v>
+        <v>305000</v>
       </c>
       <c r="L20" t="n">
-        <v>415000</v>
+        <v>279000</v>
       </c>
       <c r="M20" t="n">
-        <v>725000</v>
+        <v>365000</v>
       </c>
       <c r="N20" t="n">
-        <v>463000</v>
+        <v>299000</v>
       </c>
       <c r="O20" t="n">
-        <v>2611000</v>
+        <v>1973000</v>
       </c>
     </row>
     <row r="21">
@@ -1544,43 +1544,43 @@
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
-        <v>4031000</v>
+        <v>4428000</v>
       </c>
       <c r="D21" t="n">
-        <v>3816000</v>
+        <v>4786000</v>
       </c>
       <c r="E21" t="n">
-        <v>4070000</v>
+        <v>4714000</v>
       </c>
       <c r="F21" t="n">
-        <v>4145000</v>
+        <v>4481000</v>
       </c>
       <c r="G21" t="n">
-        <v>4219000</v>
+        <v>4602000</v>
       </c>
       <c r="H21" t="n">
-        <v>4042000</v>
+        <v>4107000</v>
       </c>
       <c r="I21" t="n">
-        <v>4455000</v>
+        <v>4429000</v>
       </c>
       <c r="J21" t="n">
-        <v>4662000</v>
+        <v>5078000</v>
       </c>
       <c r="K21" t="n">
-        <v>4577000</v>
+        <v>4707000</v>
       </c>
       <c r="L21" t="n">
-        <v>5064000</v>
+        <v>4612000</v>
       </c>
       <c r="M21" t="n">
-        <v>6840000</v>
+        <v>5714000</v>
       </c>
       <c r="N21" t="n">
-        <v>6635000</v>
+        <v>5955000</v>
       </c>
       <c r="O21" t="n">
-        <v>56556000</v>
+        <v>57613000</v>
       </c>
     </row>
   </sheetData>
@@ -1641,16 +1641,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2757000</v>
+        <v>2065000</v>
       </c>
       <c r="D2" t="n">
-        <v>2099000</v>
+        <v>1936000</v>
       </c>
       <c r="E2" t="n">
-        <v>2346000</v>
+        <v>2002000</v>
       </c>
       <c r="F2" t="n">
-        <v>3279000</v>
+        <v>2218000</v>
       </c>
     </row>
     <row r="3">
@@ -1665,16 +1665,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>438000</v>
+        <v>446000</v>
       </c>
       <c r="D3" t="n">
-        <v>751000</v>
+        <v>724000</v>
       </c>
       <c r="E3" t="n">
-        <v>800000</v>
+        <v>601000</v>
       </c>
       <c r="F3" t="n">
-        <v>721000</v>
+        <v>634000</v>
       </c>
     </row>
     <row r="4">
@@ -1689,16 +1689,16 @@
         </is>
       </c>
       <c r="C4" t="n">
+        <v>83000</v>
+      </c>
+      <c r="D4" t="n">
         <v>106000</v>
       </c>
-      <c r="D4" t="n">
-        <v>135000</v>
-      </c>
       <c r="E4" t="n">
-        <v>107000</v>
+        <v>93000</v>
       </c>
       <c r="F4" t="n">
-        <v>139000</v>
+        <v>88000</v>
       </c>
     </row>
     <row r="5">
@@ -1713,16 +1713,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>446000</v>
+        <v>339000</v>
       </c>
       <c r="D5" t="n">
-        <v>359000</v>
+        <v>346000</v>
       </c>
       <c r="E5" t="n">
-        <v>431000</v>
+        <v>328000</v>
       </c>
       <c r="F5" t="n">
-        <v>549000</v>
+        <v>394000</v>
       </c>
     </row>
     <row r="6">
@@ -1737,16 +1737,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>122000</v>
+        <v>100000</v>
       </c>
       <c r="D6" t="n">
-        <v>142000</v>
+        <v>137000</v>
       </c>
       <c r="E6" t="n">
-        <v>138000</v>
+        <v>130000</v>
       </c>
       <c r="F6" t="n">
-        <v>168000</v>
+        <v>109000</v>
       </c>
     </row>
     <row r="7">
@@ -1761,16 +1761,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>79000</v>
+        <v>59000</v>
       </c>
       <c r="D7" t="n">
-        <v>68000</v>
+        <v>65000</v>
       </c>
       <c r="E7" t="n">
-        <v>80000</v>
+        <v>64000</v>
       </c>
       <c r="F7" t="n">
-        <v>104000</v>
+        <v>69000</v>
       </c>
     </row>
     <row r="8">
@@ -1785,16 +1785,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2532000</v>
+        <v>1942000</v>
       </c>
       <c r="D8" t="n">
-        <v>2708000</v>
+        <v>1674000</v>
       </c>
       <c r="E8" t="n">
-        <v>2706000</v>
+        <v>2158000</v>
       </c>
       <c r="F8" t="n">
-        <v>3661000</v>
+        <v>2308000</v>
       </c>
     </row>
     <row r="9">
@@ -1809,16 +1809,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>573000</v>
+        <v>556000</v>
       </c>
       <c r="D9" t="n">
-        <v>842000</v>
+        <v>653000</v>
       </c>
       <c r="E9" t="n">
-        <v>688000</v>
+        <v>778000</v>
       </c>
       <c r="F9" t="n">
-        <v>973000</v>
+        <v>812000</v>
       </c>
     </row>
     <row r="10">
@@ -1833,16 +1833,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>117000</v>
+        <v>79000</v>
       </c>
       <c r="D10" t="n">
-        <v>135000</v>
+        <v>83000</v>
       </c>
       <c r="E10" t="n">
-        <v>138000</v>
+        <v>131000</v>
       </c>
       <c r="F10" t="n">
-        <v>154000</v>
+        <v>118000</v>
       </c>
     </row>
     <row r="11">
@@ -1857,16 +1857,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>484000</v>
+        <v>330000</v>
       </c>
       <c r="D11" t="n">
-        <v>440000</v>
+        <v>296000</v>
       </c>
       <c r="E11" t="n">
-        <v>437000</v>
+        <v>364000</v>
       </c>
       <c r="F11" t="n">
-        <v>604000</v>
+        <v>424000</v>
       </c>
     </row>
     <row r="12">
@@ -1881,16 +1881,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>127000</v>
+        <v>94000</v>
       </c>
       <c r="D12" t="n">
-        <v>131000</v>
+        <v>142000</v>
       </c>
       <c r="E12" t="n">
-        <v>155000</v>
+        <v>151000</v>
       </c>
       <c r="F12" t="n">
-        <v>167000</v>
+        <v>179000</v>
       </c>
     </row>
     <row r="13">
@@ -1905,16 +1905,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>82000</v>
+        <v>60000</v>
       </c>
       <c r="D13" t="n">
-        <v>80000</v>
+        <v>46000</v>
       </c>
       <c r="E13" t="n">
-        <v>73000</v>
+        <v>72000</v>
       </c>
       <c r="F13" t="n">
-        <v>104000</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="14">
@@ -1929,16 +1929,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1091000</v>
+        <v>2188000</v>
       </c>
       <c r="D14" t="n">
-        <v>1248000</v>
+        <v>1857000</v>
       </c>
       <c r="E14" t="n">
-        <v>1370000</v>
+        <v>1635000</v>
       </c>
       <c r="F14" t="n">
-        <v>1873000</v>
+        <v>2266000</v>
       </c>
     </row>
     <row r="15">
@@ -1953,16 +1953,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>234000</v>
+        <v>545000</v>
       </c>
       <c r="D15" t="n">
-        <v>441000</v>
+        <v>707000</v>
       </c>
       <c r="E15" t="n">
-        <v>511000</v>
+        <v>675000</v>
       </c>
       <c r="F15" t="n">
-        <v>536000</v>
+        <v>667000</v>
       </c>
     </row>
     <row r="16">
@@ -1977,16 +1977,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>37000</v>
+        <v>96000</v>
       </c>
       <c r="D16" t="n">
-        <v>74000</v>
+        <v>81000</v>
       </c>
       <c r="E16" t="n">
-        <v>73000</v>
+        <v>87000</v>
       </c>
       <c r="F16" t="n">
-        <v>85000</v>
+        <v>109000</v>
       </c>
     </row>
     <row r="17">
@@ -2001,16 +2001,16 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>185000</v>
+        <v>354000</v>
       </c>
       <c r="D17" t="n">
-        <v>216000</v>
+        <v>293000</v>
       </c>
       <c r="E17" t="n">
-        <v>229000</v>
+        <v>301000</v>
       </c>
       <c r="F17" t="n">
-        <v>373000</v>
+        <v>400000</v>
       </c>
     </row>
     <row r="18">
@@ -2025,16 +2025,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>52000</v>
+        <v>104000</v>
       </c>
       <c r="D18" t="n">
-        <v>93000</v>
+        <v>137000</v>
       </c>
       <c r="E18" t="n">
-        <v>103000</v>
+        <v>134000</v>
       </c>
       <c r="F18" t="n">
-        <v>113000</v>
+        <v>123000</v>
       </c>
     </row>
     <row r="19">
@@ -2049,16 +2049,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>28000</v>
+        <v>57000</v>
       </c>
       <c r="D19" t="n">
-        <v>41000</v>
+        <v>62000</v>
       </c>
       <c r="E19" t="n">
-        <v>40000</v>
+        <v>56000</v>
       </c>
       <c r="F19" t="n">
-        <v>57000</v>
+        <v>62000</v>
       </c>
     </row>
     <row r="20">
@@ -2073,16 +2073,16 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1412000</v>
+        <v>2783000</v>
       </c>
       <c r="D20" t="n">
-        <v>1312000</v>
+        <v>2225000</v>
       </c>
       <c r="E20" t="n">
-        <v>1777000</v>
+        <v>2491000</v>
       </c>
       <c r="F20" t="n">
-        <v>3065000</v>
+        <v>3313000</v>
       </c>
     </row>
     <row r="21">
@@ -2097,16 +2097,16 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>381000</v>
+        <v>582000</v>
       </c>
       <c r="D21" t="n">
-        <v>422000</v>
+        <v>725000</v>
       </c>
       <c r="E21" t="n">
-        <v>650000</v>
+        <v>899000</v>
       </c>
       <c r="F21" t="n">
-        <v>657000</v>
+        <v>754000</v>
       </c>
     </row>
     <row r="22">
@@ -2121,16 +2121,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>54000</v>
+        <v>116000</v>
       </c>
       <c r="D22" t="n">
-        <v>79000</v>
+        <v>118000</v>
       </c>
       <c r="E22" t="n">
-        <v>110000</v>
+        <v>156000</v>
       </c>
       <c r="F22" t="n">
-        <v>126000</v>
+        <v>133000</v>
       </c>
     </row>
     <row r="23">
@@ -2145,16 +2145,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>243000</v>
+        <v>483000</v>
       </c>
       <c r="D23" t="n">
-        <v>231000</v>
+        <v>355000</v>
       </c>
       <c r="E23" t="n">
-        <v>305000</v>
+        <v>432000</v>
       </c>
       <c r="F23" t="n">
-        <v>510000</v>
+        <v>507000</v>
       </c>
     </row>
     <row r="24">
@@ -2169,16 +2169,16 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>86000</v>
+        <v>148000</v>
       </c>
       <c r="D24" t="n">
-        <v>96000</v>
+        <v>140000</v>
       </c>
       <c r="E24" t="n">
-        <v>126000</v>
+        <v>163000</v>
       </c>
       <c r="F24" t="n">
-        <v>102000</v>
+        <v>163000</v>
       </c>
     </row>
     <row r="25">
@@ -2193,16 +2193,16 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>44000</v>
+        <v>84000</v>
       </c>
       <c r="D25" t="n">
-        <v>44000</v>
+        <v>70000</v>
       </c>
       <c r="E25" t="n">
-        <v>52000</v>
+        <v>77000</v>
       </c>
       <c r="F25" t="n">
-        <v>91000</v>
+        <v>84000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>